<commit_message>
Update division of work
</commit_message>
<xml_diff>
--- a/PCCV.xlsx
+++ b/PCCV.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HKII_4\Android\KT\BTLMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A408CA8F-614C-4C06-BB66-33F857A78AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8CEFAD1-882F-4991-99CC-ED5BD94C5AA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A879458F-AEFE-4FBF-B135-619A5E44A0ED}"/>
   </bookViews>
@@ -101,32 +101,37 @@
     <t>Mô tả chi tiết</t>
   </si>
   <si>
-    <t>Model: Tạo lớp Room với các trường dữ liệu: Mã, Tên, Giá, Tình trạng (Boolean/String), Người thuê, SĐT.Data Singleton: Tạo một Class chứa public static List&lt;Room&gt; roomList và add sẵn 5-10 dữ liệu mẫu (Dummy data). Việc này giúp Thành viên 2 có cái để hiển thị lên RecyclerView ngay lập tức mà không cần đợi Thành viên 3 làm xong chức năng Thêm.Git Manager: Khởi tạo Repo, tạo 3 nhánh phụ cho 3 người còn lại merge vào.</t>
-  </si>
-  <si>
-    <t>Layout: Thiết kế item_room.xml (CardView) và activity_main.xml (RecyclerView).Adapter: Viết RoomAdapter. Quan trọng nhất là logic onBindViewHolder:Nếu status == "Đã thuê" -&gt; Set background/Text màu Đỏ.Nếu status == "Còn trống" -&gt; Set background/Text màu Xanh.Action: Bắt sự kiện Click vào item để mở màn hình Sửa và LongClick để Xóa.</t>
+    <t>Khởi tạo project, tạo model, push base, thực hiện chức năng tìm kiếm</t>
+  </si>
+  <si>
+    <t>Thực hiện chức năng sửa thông tin và xác nhận xóa.</t>
+  </si>
+  <si>
+    <t>Thực hiện việc xây dựng màn hình thêm mới và bắt lỗi nhập liệu</t>
+  </si>
+  <si>
+    <t>Thực hiện chức năng đọc, hiển thị danh sách, phân công công việc</t>
+  </si>
+  <si>
+    <t>Update: Tạo ActivityEditRoom. Khi nhấn vào item, hiển thị dữ liệu của phòng đã nhấn vào các EditText để người dùng sửa. Sau đó cập nhật lại đúng vị trí (index) đó trong List.
+Delete: Xử lý AlertDialog khi nhấn button Remove. 
+Nếu người dùng chọn "Yes", thực hiện roomList.remove(position) và cập nhật lại giao diện.</t>
   </si>
   <si>
     <t>Layout: Tạo ActivityAddRoom với các EditText.
-Validate: Kiểm tra nhanh: Tên phòng không trống, Giá phải là số.
-Logic: Nhấn "Lưu" thì roomList.add(newRoom) và gọi adapter.notifyDataSetChanged() hoặc dùng Intent trả kết quả về màn hình chính.</t>
-  </si>
-  <si>
-    <t>Khởi tạo project, tạo model, push base, thực hiện chức năng tìm kiếm</t>
-  </si>
-  <si>
-    <t>Thiết kế giao diện, hiển thị danh sách, phân công công việc</t>
-  </si>
-  <si>
-    <t>Thực hiện chức năng sửa thông tin và xác nhận xóa.</t>
-  </si>
-  <si>
-    <t>Thực hiện việc xây dựng màn hình thêm mới và bắt lỗi nhập liệu</t>
-  </si>
-  <si>
-    <t>Update: Tạo ActivityEditRoom. Khi nhấn vào item, hiển thị dữ liệu cũ của phòng đã nhấn vào các EditText để người dùng sửa. Sau đó cập nhật lại đúng vị trí (index) đó trong List.
-Delete: Xử lý AlertDialog khi nhấn giữ item. 
-Nếu người dùng chọn "Yes", thực hiện roomList.remove(position) và cập nhật lại giao diện.</t>
+Validate: Kiểm tra nhanh: Tên phòng không trống, giá phải là số.
+Logic: Nhấn nút Add thì gọi adapter hoặc dùng Intent trả kết quả về màn hình RecycleView.</t>
+  </si>
+  <si>
+    <t>Layout: Thiết kế item_room.xml (CardView) và activity_main.xml (RecyclerView).Adapter: Viết RoomAdapter. 
+Action: Bắt sự kiện click vào item để hiện thông tin sửa và nhấn nút remove để hiện AlertDialog.
+Viết excel phân chia công việc.</t>
+  </si>
+  <si>
+    <t>Model: Tạo lớp Room với các trường dữ liệu: Mã, tên, giá, tình trạng , người thuê, SĐT.
+Data Singleton: Tạo một Class chứa public static List&lt;Room&gt; roomList. 
+Git Manager: Khởi tạo project, github, push base, gửi thông tin lên link excel.
+Search: Gõ vào thanh search để tìm item trong RecycleView.</t>
   </si>
 </sst>
 </file>
@@ -303,7 +308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -339,34 +344,13 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -374,6 +358,24 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -714,30 +716,31 @@
   <cols>
     <col min="1" max="1" width="21.7109375" style="1" customWidth="1"/>
     <col min="2" max="3" width="26.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="34.85546875" style="1" customWidth="1"/>
-    <col min="5" max="6" width="69.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="31.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="38.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="77" style="1" customWidth="1"/>
+    <col min="6" max="6" width="40" style="1" customWidth="1"/>
+    <col min="7" max="7" width="35.28515625" style="1" customWidth="1"/>
     <col min="8" max="9" width="9.140625" style="1"/>
     <col min="10" max="10" width="18.42578125" style="1" customWidth="1"/>
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
     </row>
     <row r="2" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="20"/>
+      <c r="B2" s="23"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="8" t="s">
@@ -757,11 +760,11 @@
       <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="17"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="20"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
@@ -805,11 +808,11 @@
       <c r="C6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="23" t="s">
+      <c r="D6" s="16" t="s">
         <v>23</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -824,16 +827,16 @@
       <c r="C7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" s="14"/>
+      <c r="D7" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="13"/>
       <c r="G7" s="6"/>
     </row>
-    <row r="8" spans="1:7" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="139.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
         <v>3</v>
       </c>
@@ -843,13 +846,13 @@
       <c r="C8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="14"/>
+      <c r="D8" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="13"/>
       <c r="G8" s="6"/>
     </row>
     <row r="9" spans="1:7" ht="138.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -862,23 +865,23 @@
       <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="24" t="s">
+      <c r="D9" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="14"/>
+      <c r="E9" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="13"/>
       <c r="G9" s="6"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="21"/>
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>